<commit_message>
Update examples and tests
Got the Helsley data from West Coast example added and got the code to pass all the tests as well as update tests for new stuff.
</commit_message>
<xml_diff>
--- a/tests/test_convert/testing_files/main_dir/mwtab_ms_conversion_directives_compare.xlsx
+++ b/tests/test_convert/testing_files/main_dir/mwtab_ms_conversion_directives_compare.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="137">
   <si>
     <t>#tags</t>
   </si>
@@ -145,6 +145,21 @@
     <t>INSTRUMENT_NAME</t>
   </si>
   <si>
+    <t>FLOW_GRADIENT</t>
+  </si>
+  <si>
+    <t>FLOW_RATE</t>
+  </si>
+  <si>
+    <t>COLUMN_TEMPERATURE</t>
+  </si>
+  <si>
+    <t>SOLVENT_A</t>
+  </si>
+  <si>
+    <t>SOLVENT_B</t>
+  </si>
+  <si>
     <t>#ANALYSIS.id</t>
   </si>
   <si>
@@ -268,6 +283,21 @@
     <t>chromatography_instrument_name</t>
   </si>
   <si>
+    <t>flow_gradient</t>
+  </si>
+  <si>
+    <t>flow_rate</t>
+  </si>
+  <si>
+    <t>column_temperature</t>
+  </si>
+  <si>
+    <t>solvent_a</t>
+  </si>
+  <si>
+    <t>solvent_b</t>
+  </si>
+  <si>
     <t>MS</t>
   </si>
   <si>
@@ -313,6 +343,36 @@
     <t>False</t>
   </si>
   <si>
+    <t>#.fill_headers</t>
+  </si>
+  <si>
+    <t>#.fields_to_headers</t>
+  </si>
+  <si>
+    <t>#.table</t>
+  </si>
+  <si>
+    <t>project</t>
+  </si>
+  <si>
+    <t>study</t>
+  </si>
+  <si>
+    <t>entity</t>
+  </si>
+  <si>
+    <t>section</t>
+  </si>
+  <si>
+    <t>protocol</t>
+  </si>
+  <si>
+    <t>#.for_each</t>
+  </si>
+  <si>
+    <t>measurement</t>
+  </si>
+  <si>
     <t>*#.headers</t>
   </si>
   <si>
@@ -322,31 +382,16 @@
     <t>"Metabolite"=assignment</t>
   </si>
   <si>
-    <t>#.fields_to_headers</t>
-  </si>
-  <si>
-    <t>#.table</t>
-  </si>
-  <si>
-    <t>project</t>
-  </si>
-  <si>
-    <t>study</t>
-  </si>
-  <si>
-    <t>entity</t>
-  </si>
-  <si>
-    <t>section</t>
-  </si>
-  <si>
-    <t>protocol</t>
-  </si>
-  <si>
-    <t>#.for_each</t>
-  </si>
-  <si>
-    <t>measurement</t>
+    <t>#.test</t>
+  </si>
+  <si>
+    <t>type=subject</t>
+  </si>
+  <si>
+    <t>type=collection</t>
+  </si>
+  <si>
+    <t>machine_type=MS</t>
   </si>
   <si>
     <t>*#.optional_headers</t>
@@ -358,18 +403,6 @@
     <t>"Metabolite"=assignment,"sample_id"=entity.id</t>
   </si>
   <si>
-    <t>#.test</t>
-  </si>
-  <si>
-    <t>type=subject</t>
-  </si>
-  <si>
-    <t>type=collection</t>
-  </si>
-  <si>
-    <t>machine_type=MS</t>
-  </si>
-  <si>
     <t>*#.sort_by</t>
   </si>
   <si>
@@ -382,13 +415,13 @@
     <t>ascending</t>
   </si>
   <si>
+    <t>type=treatment</t>
+  </si>
+  <si>
+    <t>type=sample_prep</t>
+  </si>
+  <si>
     <t>matrix</t>
-  </si>
-  <si>
-    <t>type=treatment</t>
-  </si>
-  <si>
-    <t>type=sample_prep</t>
   </si>
   <si>
     <t>#.values_to_str</t>
@@ -723,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -734,10 +767,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -745,10 +778,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -756,10 +789,10 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -767,10 +800,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -781,10 +814,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -792,10 +825,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -806,16 +839,16 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -823,16 +856,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E10" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F10" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -840,16 +873,16 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F11" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -857,16 +890,16 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -874,16 +907,16 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D13" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E13" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -891,16 +924,16 @@
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E14" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F14" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -908,16 +941,16 @@
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E15" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F15" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -925,16 +958,16 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F16" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -942,16 +975,16 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F17" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -959,16 +992,16 @@
         <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F18" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -979,16 +1012,16 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E20" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F20" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -996,16 +1029,16 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1013,16 +1046,16 @@
         <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D22" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E22" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1030,16 +1063,16 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1047,16 +1080,16 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D24" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E24" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F24" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1064,16 +1097,16 @@
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E25" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1081,16 +1114,16 @@
         <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D26" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E26" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1098,16 +1131,16 @@
         <v>13</v>
       </c>
       <c r="C27" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F27" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1115,16 +1148,16 @@
         <v>17</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D28" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F28" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1132,16 +1165,16 @@
         <v>18</v>
       </c>
       <c r="C29" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D29" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F29" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1152,19 +1185,19 @@
         <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E31" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F31" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G31" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1172,19 +1205,19 @@
         <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E32" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G32" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -1192,19 +1225,19 @@
         <v>21</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D33" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E33" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G33" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -1212,19 +1245,19 @@
         <v>22</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E34" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -1235,13 +1268,13 @@
         <v>23</v>
       </c>
       <c r="C36" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D36" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -1249,13 +1282,13 @@
         <v>24</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E37" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -1266,19 +1299,19 @@
         <v>25</v>
       </c>
       <c r="C39" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D39" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E39" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F39" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G39" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -1286,19 +1319,19 @@
         <v>26</v>
       </c>
       <c r="C40" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D40" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F40" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G40" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -1306,19 +1339,19 @@
         <v>27</v>
       </c>
       <c r="C41" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D41" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E41" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F41" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G41" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -1326,19 +1359,19 @@
         <v>28</v>
       </c>
       <c r="C42" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D42" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E42" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F42" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G42" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -1346,19 +1379,19 @@
         <v>29</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D43" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E43" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F43" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="G43" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -1369,31 +1402,31 @@
         <v>30</v>
       </c>
       <c r="C45" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D45" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E45" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F45" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G45" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="H45" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="I45" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="J45" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="K45" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -1401,31 +1434,31 @@
         <v>31</v>
       </c>
       <c r="C46" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D46" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E46" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F46" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="G46" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H46" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I46" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J46" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="K46" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -1433,31 +1466,31 @@
         <v>32</v>
       </c>
       <c r="C47" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D47" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E47" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F47" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G47" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H47" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I47" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J47" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="K47" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -1465,31 +1498,31 @@
         <v>33</v>
       </c>
       <c r="C48" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D48" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E48" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F48" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G48" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H48" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I48" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J48" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="K48" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -1500,31 +1533,31 @@
         <v>34</v>
       </c>
       <c r="C50" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D50" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E50" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F50" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G50" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="H50" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="I50" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="J50" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="K50" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -1532,31 +1565,31 @@
         <v>35</v>
       </c>
       <c r="C51" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D51" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E51" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F51" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="G51" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="H51" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I51" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J51" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="K51" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -1564,31 +1597,31 @@
         <v>36</v>
       </c>
       <c r="C52" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D52" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E52" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F52" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G52" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="H52" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I52" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J52" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="K52" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -1596,31 +1629,31 @@
         <v>37</v>
       </c>
       <c r="C53" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D53" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E53" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="F53" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G53" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="H53" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="I53" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J53" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="K53" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -1631,19 +1664,19 @@
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D55" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E55" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F55" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G55" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -1651,19 +1684,19 @@
         <v>39</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D56" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="E56" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F56" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G56" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -1671,19 +1704,19 @@
         <v>40</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D57" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E57" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F57" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G57" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -1691,19 +1724,19 @@
         <v>41</v>
       </c>
       <c r="C58" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D58" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E58" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F58" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G58" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -1711,399 +1744,508 @@
         <v>42</v>
       </c>
       <c r="C59" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D59" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E59" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F59" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G59" t="s">
-        <v>95</v>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11">
+      <c r="B60" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" t="s">
+        <v>89</v>
+      </c>
+      <c r="D60" t="s">
+        <v>107</v>
+      </c>
+      <c r="E60" t="s">
+        <v>116</v>
+      </c>
+      <c r="F60" t="s">
+        <v>125</v>
+      </c>
+      <c r="G60" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" t="s">
-        <v>0</v>
-      </c>
       <c r="B61" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C61" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>94</v>
+        <v>107</v>
+      </c>
+      <c r="E61" t="s">
+        <v>116</v>
+      </c>
+      <c r="F61" t="s">
+        <v>125</v>
+      </c>
+      <c r="G61" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="62" spans="1:11">
       <c r="B62" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C62" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D62" t="s">
-        <v>95</v>
+        <v>107</v>
+      </c>
+      <c r="E62" t="s">
+        <v>116</v>
+      </c>
+      <c r="F62" t="s">
+        <v>125</v>
+      </c>
+      <c r="G62" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11">
+      <c r="B63" t="s">
+        <v>46</v>
+      </c>
+      <c r="C63" t="s">
+        <v>92</v>
+      </c>
+      <c r="D63" t="s">
+        <v>107</v>
+      </c>
+      <c r="E63" t="s">
+        <v>116</v>
+      </c>
+      <c r="F63" t="s">
+        <v>125</v>
+      </c>
+      <c r="G63" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
+        <v>47</v>
+      </c>
+      <c r="C64" t="s">
+        <v>93</v>
+      </c>
+      <c r="D64" t="s">
+        <v>107</v>
+      </c>
+      <c r="E64" t="s">
+        <v>116</v>
+      </c>
+      <c r="F64" t="s">
+        <v>125</v>
+      </c>
+      <c r="G64" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11">
+      <c r="A66" t="s">
         <v>0</v>
       </c>
-      <c r="B64" t="s">
-        <v>45</v>
-      </c>
-      <c r="C64" t="s">
-        <v>61</v>
-      </c>
-      <c r="D64" t="s">
-        <v>96</v>
-      </c>
-      <c r="E64" t="s">
-        <v>103</v>
-      </c>
-      <c r="F64" t="s">
-        <v>114</v>
-      </c>
-      <c r="G64" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11">
-      <c r="B65" t="s">
-        <v>42</v>
-      </c>
-      <c r="C65" t="s">
-        <v>85</v>
-      </c>
-      <c r="D65" t="s">
-        <v>97</v>
-      </c>
-      <c r="E65" t="s">
-        <v>108</v>
-      </c>
-      <c r="F65" t="s">
-        <v>117</v>
-      </c>
-      <c r="G65" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11">
       <c r="B66" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="D66" t="s">
-        <v>97</v>
-      </c>
-      <c r="E66" t="s">
-        <v>108</v>
-      </c>
-      <c r="F66" t="s">
-        <v>117</v>
-      </c>
-      <c r="G66" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="67" spans="1:11">
       <c r="B67" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C67" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D67" t="s">
-        <v>97</v>
-      </c>
-      <c r="E67" t="s">
-        <v>108</v>
-      </c>
-      <c r="F67" t="s">
-        <v>117</v>
-      </c>
-      <c r="G67" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11">
+      <c r="A69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" t="s">
+        <v>50</v>
+      </c>
+      <c r="C69" t="s">
+        <v>66</v>
+      </c>
+      <c r="D69" t="s">
+        <v>106</v>
+      </c>
+      <c r="E69" t="s">
+        <v>111</v>
+      </c>
+      <c r="F69" t="s">
+        <v>122</v>
+      </c>
+      <c r="G69" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11">
+      <c r="B70" t="s">
+        <v>42</v>
+      </c>
+      <c r="C70" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="68" spans="1:11">
-      <c r="B68" t="s">
-        <v>48</v>
-      </c>
-      <c r="C68" t="s">
-        <v>69</v>
-      </c>
-      <c r="D68" t="s">
-        <v>98</v>
-      </c>
-      <c r="E68" t="s">
-        <v>108</v>
-      </c>
-      <c r="F68" t="s">
-        <v>117</v>
-      </c>
-      <c r="G68" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11">
-      <c r="B69" t="s">
-        <v>49</v>
-      </c>
-      <c r="C69" t="s">
-        <v>88</v>
-      </c>
-      <c r="D69" t="s">
-        <v>97</v>
-      </c>
-      <c r="E69" t="s">
-        <v>108</v>
-      </c>
-      <c r="F69" t="s">
-        <v>117</v>
-      </c>
-      <c r="G69" t="s">
-        <v>95</v>
+      <c r="D70" t="s">
+        <v>107</v>
+      </c>
+      <c r="E70" t="s">
+        <v>116</v>
+      </c>
+      <c r="F70" t="s">
+        <v>125</v>
+      </c>
+      <c r="G70" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="71" spans="1:11">
-      <c r="A71" t="s">
-        <v>0</v>
-      </c>
       <c r="B71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C71" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="D71" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E71" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="F71" t="s">
-        <v>94</v>
+        <v>125</v>
+      </c>
+      <c r="G71" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="72" spans="1:11">
       <c r="B72" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C72" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D72" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E72" t="s">
+        <v>116</v>
+      </c>
+      <c r="F72" t="s">
+        <v>125</v>
+      </c>
+      <c r="G72" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11">
+      <c r="B73" t="s">
+        <v>53</v>
+      </c>
+      <c r="C73" t="s">
+        <v>74</v>
+      </c>
+      <c r="D73" t="s">
+        <v>108</v>
+      </c>
+      <c r="E73" t="s">
+        <v>116</v>
+      </c>
+      <c r="F73" t="s">
+        <v>125</v>
+      </c>
+      <c r="G73" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11">
+      <c r="B74" t="s">
+        <v>54</v>
+      </c>
+      <c r="C74" t="s">
+        <v>98</v>
+      </c>
+      <c r="D74" t="s">
+        <v>107</v>
+      </c>
+      <c r="E74" t="s">
+        <v>116</v>
+      </c>
+      <c r="F74" t="s">
+        <v>125</v>
+      </c>
+      <c r="G74" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
+        <v>55</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76" t="s">
+        <v>106</v>
+      </c>
+      <c r="E76" t="s">
+        <v>111</v>
+      </c>
+      <c r="F76" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11">
+      <c r="B77" t="s">
+        <v>56</v>
+      </c>
+      <c r="C77" t="s">
+        <v>99</v>
+      </c>
+      <c r="D77" t="s">
+        <v>107</v>
+      </c>
+      <c r="E77" t="s">
+        <v>118</v>
+      </c>
+      <c r="F77" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11">
+      <c r="A79" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" t="s">
+        <v>55</v>
+      </c>
+      <c r="C79" t="s">
+        <v>100</v>
+      </c>
+      <c r="D79" t="s">
+        <v>109</v>
+      </c>
+      <c r="E79" t="s">
+        <v>119</v>
+      </c>
+      <c r="F79" t="s">
+        <v>106</v>
+      </c>
+      <c r="G79" t="s">
+        <v>129</v>
+      </c>
+      <c r="H79" t="s">
+        <v>131</v>
+      </c>
+      <c r="I79" t="s">
+        <v>111</v>
+      </c>
+      <c r="J79" t="s">
+        <v>104</v>
+      </c>
+      <c r="K79" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11">
+      <c r="B80" t="s">
+        <v>57</v>
+      </c>
+      <c r="C80" t="s">
+        <v>101</v>
+      </c>
+      <c r="E80" t="s">
+        <v>120</v>
+      </c>
+      <c r="F80" t="s">
+        <v>107</v>
+      </c>
+      <c r="G80" t="s">
+        <v>101</v>
+      </c>
+      <c r="H80" t="s">
+        <v>132</v>
+      </c>
+      <c r="I80" t="s">
+        <v>118</v>
+      </c>
+      <c r="J80" t="s">
+        <v>135</v>
+      </c>
+      <c r="K80" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12">
+      <c r="A82" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" t="s">
+        <v>55</v>
+      </c>
+      <c r="C82" t="s">
+        <v>100</v>
+      </c>
+      <c r="D82" t="s">
+        <v>109</v>
+      </c>
+      <c r="E82" t="s">
+        <v>119</v>
+      </c>
+      <c r="F82" t="s">
+        <v>126</v>
+      </c>
+      <c r="G82" t="s">
+        <v>106</v>
+      </c>
+      <c r="H82" t="s">
+        <v>129</v>
+      </c>
+      <c r="I82" t="s">
+        <v>131</v>
+      </c>
+      <c r="J82" t="s">
+        <v>111</v>
+      </c>
+      <c r="K82" t="s">
+        <v>104</v>
+      </c>
+      <c r="L82" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12">
+      <c r="B83" t="s">
+        <v>58</v>
+      </c>
+      <c r="C83" t="s">
+        <v>101</v>
+      </c>
+      <c r="E83" t="s">
+        <v>121</v>
+      </c>
+      <c r="F83" t="s">
+        <v>127</v>
+      </c>
+      <c r="G83" t="s">
+        <v>107</v>
+      </c>
+      <c r="H83" t="s">
+        <v>101</v>
+      </c>
+      <c r="I83" t="s">
+        <v>132</v>
+      </c>
+      <c r="J83" t="s">
+        <v>118</v>
+      </c>
+      <c r="K83" t="s">
+        <v>135</v>
+      </c>
+      <c r="L83" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
+        <v>55</v>
+      </c>
+      <c r="C85" t="s">
+        <v>102</v>
+      </c>
+      <c r="D85" t="s">
         <v>110</v>
       </c>
-      <c r="F72" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11">
-      <c r="A74" t="s">
-        <v>0</v>
-      </c>
-      <c r="B74" t="s">
-        <v>50</v>
-      </c>
-      <c r="C74" t="s">
-        <v>90</v>
-      </c>
-      <c r="D74" t="s">
-        <v>99</v>
-      </c>
-      <c r="E74" t="s">
-        <v>96</v>
-      </c>
-      <c r="F74" t="s">
+      <c r="E85" t="s">
+        <v>109</v>
+      </c>
+      <c r="F85" t="s">
+        <v>119</v>
+      </c>
+      <c r="G85" t="s">
+        <v>106</v>
+      </c>
+      <c r="H85" t="s">
+        <v>129</v>
+      </c>
+      <c r="I85" t="s">
+        <v>131</v>
+      </c>
+      <c r="J85" t="s">
+        <v>111</v>
+      </c>
+      <c r="K85" t="s">
+        <v>104</v>
+      </c>
+      <c r="L85" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12">
+      <c r="B86" t="s">
+        <v>59</v>
+      </c>
+      <c r="C86" t="s">
+        <v>103</v>
+      </c>
+      <c r="D86" t="s">
+        <v>107</v>
+      </c>
+      <c r="F86" t="s">
+        <v>128</v>
+      </c>
+      <c r="G86" t="s">
+        <v>108</v>
+      </c>
+      <c r="H86" t="s">
+        <v>101</v>
+      </c>
+      <c r="I86" t="s">
+        <v>132</v>
+      </c>
+      <c r="J86" t="s">
         <v>118</v>
       </c>
-      <c r="G74" t="s">
-        <v>120</v>
-      </c>
-      <c r="H74" t="s">
-        <v>103</v>
-      </c>
-      <c r="I74" t="s">
-        <v>94</v>
-      </c>
-      <c r="J74" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11">
-      <c r="B75" t="s">
-        <v>52</v>
-      </c>
-      <c r="C75" t="s">
-        <v>91</v>
-      </c>
-      <c r="D75" t="s">
-        <v>100</v>
-      </c>
-      <c r="E75" t="s">
-        <v>97</v>
-      </c>
-      <c r="F75" t="s">
-        <v>91</v>
-      </c>
-      <c r="G75" t="s">
-        <v>121</v>
-      </c>
-      <c r="H75" t="s">
-        <v>110</v>
-      </c>
-      <c r="I75" t="s">
-        <v>122</v>
-      </c>
-      <c r="J75" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11">
-      <c r="A77" t="s">
-        <v>0</v>
-      </c>
-      <c r="B77" t="s">
-        <v>50</v>
-      </c>
-      <c r="C77" t="s">
-        <v>90</v>
-      </c>
-      <c r="D77" t="s">
-        <v>99</v>
-      </c>
-      <c r="E77" t="s">
-        <v>111</v>
-      </c>
-      <c r="F77" t="s">
-        <v>96</v>
-      </c>
-      <c r="G77" t="s">
-        <v>118</v>
-      </c>
-      <c r="H77" t="s">
-        <v>120</v>
-      </c>
-      <c r="I77" t="s">
-        <v>103</v>
-      </c>
-      <c r="J77" t="s">
-        <v>94</v>
-      </c>
-      <c r="K77" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11">
-      <c r="B78" t="s">
-        <v>53</v>
-      </c>
-      <c r="C78" t="s">
-        <v>91</v>
-      </c>
-      <c r="D78" t="s">
-        <v>101</v>
-      </c>
-      <c r="E78" t="s">
-        <v>112</v>
-      </c>
-      <c r="F78" t="s">
-        <v>97</v>
-      </c>
-      <c r="G78" t="s">
-        <v>91</v>
-      </c>
-      <c r="H78" t="s">
-        <v>121</v>
-      </c>
-      <c r="I78" t="s">
-        <v>110</v>
-      </c>
-      <c r="J78" t="s">
-        <v>122</v>
-      </c>
-      <c r="K78" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11">
-      <c r="A80" t="s">
-        <v>0</v>
-      </c>
-      <c r="B80" t="s">
-        <v>50</v>
-      </c>
-      <c r="C80" t="s">
-        <v>92</v>
-      </c>
-      <c r="D80" t="s">
-        <v>102</v>
-      </c>
-      <c r="E80" t="s">
-        <v>99</v>
-      </c>
-      <c r="F80" t="s">
-        <v>96</v>
-      </c>
-      <c r="G80" t="s">
-        <v>118</v>
-      </c>
-      <c r="H80" t="s">
-        <v>120</v>
-      </c>
-      <c r="I80" t="s">
-        <v>103</v>
-      </c>
-      <c r="J80" t="s">
-        <v>94</v>
-      </c>
-      <c r="K80" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="81" spans="2:11">
-      <c r="B81" t="s">
-        <v>54</v>
-      </c>
-      <c r="C81" t="s">
-        <v>93</v>
-      </c>
-      <c r="D81" t="s">
-        <v>97</v>
-      </c>
-      <c r="E81" t="s">
-        <v>113</v>
-      </c>
-      <c r="F81" t="s">
-        <v>98</v>
-      </c>
-      <c r="G81" t="s">
-        <v>91</v>
-      </c>
-      <c r="H81" t="s">
-        <v>121</v>
-      </c>
-      <c r="I81" t="s">
-        <v>110</v>
-      </c>
-      <c r="J81" t="s">
-        <v>122</v>
-      </c>
-      <c r="K81" t="s">
-        <v>97</v>
+      <c r="K86" t="s">
+        <v>135</v>
+      </c>
+      <c r="L86" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>